<commit_message>
Added GitHub hyperlink - Kumar Prakhar
</commit_message>
<xml_diff>
--- a/Java_Selenium_Batch_1_Capstone_Project.xlsx
+++ b/Java_Selenium_Batch_1_Capstone_Project.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e7c05477d0ad59ef/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\GitDemo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{80320C52-5062-4567-A899-5F3D79A0AD1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAD07335-B099-4EA2-B167-9507F92E34E6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C66033-8A35-4C89-B1DD-35C5676289FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{124B4E3D-77E1-470B-83A3-A7978E63010D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>S No</t>
   </si>
@@ -172,13 +172,16 @@
   </si>
   <si>
     <t>Capstone_Project_Git_Link</t>
+  </si>
+  <si>
+    <t>https://github.com/KumarPrakhar12/FlightBookingAutomation.git</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,6 +205,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -282,10 +293,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -305,8 +317,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -983,7 +997,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="3">
         <v>35</v>
       </c>
@@ -994,7 +1008,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="3">
         <v>36</v>
       </c>
@@ -1005,7 +1019,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="3">
         <v>37</v>
       </c>
@@ -1016,7 +1030,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="3">
         <v>38</v>
       </c>
@@ -1027,7 +1041,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="3">
         <v>40</v>
       </c>
@@ -1038,7 +1052,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="3">
         <v>41</v>
       </c>
@@ -1049,7 +1063,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="3">
         <v>42</v>
       </c>
@@ -1060,7 +1074,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="3">
         <v>43</v>
       </c>
@@ -1071,7 +1085,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="3">
         <v>44</v>
       </c>
@@ -1081,8 +1095,11 @@
       <c r="C41" s="8" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D41" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="3">
         <v>46</v>
       </c>
@@ -1093,7 +1110,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="3">
         <v>47</v>
       </c>
@@ -1105,6 +1122,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D41" r:id="rId1" xr:uid="{0167339C-FC05-4449-82D7-47A419CB0119}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Addede my Github repo Link-Sachin
</commit_message>
<xml_diff>
--- a/Java_Selenium_Batch_1_Capstone_Project.xlsx
+++ b/Java_Selenium_Batch_1_Capstone_Project.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e7c05477d0ad59ef/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sachin\Desktop\GitDemoRep\GitDemo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{80320C52-5062-4567-A899-5F3D79A0AD1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAD07335-B099-4EA2-B167-9507F92E34E6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82283DAF-2A36-4B7D-AE71-DC5D46A301F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{124B4E3D-77E1-470B-83A3-A7978E63010D}"/>
+    <workbookView xWindow="1428" yWindow="1428" windowWidth="17280" windowHeight="8880" xr2:uid="{124B4E3D-77E1-470B-83A3-A7978E63010D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,21 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>S No</t>
   </si>
@@ -172,13 +163,16 @@
   </si>
   <si>
     <t>Capstone_Project_Git_Link</t>
+  </si>
+  <si>
+    <t>https://github.com/sachind0143/CapstoneProject</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,6 +196,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -282,10 +284,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -305,8 +308,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -620,15 +625,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C56D031-3353-4F8C-88A6-A34A4269BBE8}">
   <dimension ref="A1:D43"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.90625" customWidth="1"/>
-    <col min="2" max="2" width="14.90625" customWidth="1"/>
-    <col min="3" max="3" width="37.54296875" customWidth="1"/>
-    <col min="4" max="4" width="25.81640625" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" customWidth="1"/>
+    <col min="3" max="3" width="37.5546875" customWidth="1"/>
+    <col min="4" max="4" width="42.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -642,7 +647,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -653,7 +658,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -664,7 +669,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -675,7 +680,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -686,7 +691,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -697,7 +702,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -708,7 +713,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>8</v>
       </c>
@@ -719,7 +724,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>9</v>
       </c>
@@ -730,7 +735,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>10</v>
       </c>
@@ -741,7 +746,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>11</v>
       </c>
@@ -752,7 +757,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>13</v>
       </c>
@@ -763,7 +768,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>14</v>
       </c>
@@ -774,7 +779,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>15</v>
       </c>
@@ -785,7 +790,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>16</v>
       </c>
@@ -796,7 +801,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>17</v>
       </c>
@@ -807,7 +812,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>18</v>
       </c>
@@ -818,7 +823,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>19</v>
       </c>
@@ -829,7 +834,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>20</v>
       </c>
@@ -840,7 +845,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>21</v>
       </c>
@@ -851,7 +856,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>23</v>
       </c>
@@ -862,7 +867,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>24</v>
       </c>
@@ -873,7 +878,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>25</v>
       </c>
@@ -884,7 +889,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>26</v>
       </c>
@@ -895,7 +900,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>27</v>
       </c>
@@ -906,7 +911,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>28</v>
       </c>
@@ -917,7 +922,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>29</v>
       </c>
@@ -928,7 +933,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>30</v>
       </c>
@@ -939,7 +944,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>31</v>
       </c>
@@ -950,7 +955,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>32</v>
       </c>
@@ -961,7 +966,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>33</v>
       </c>
@@ -972,7 +977,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>34</v>
       </c>
@@ -983,7 +988,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>35</v>
       </c>
@@ -994,7 +999,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="3">
         <v>36</v>
       </c>
@@ -1005,7 +1010,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
         <v>37</v>
       </c>
@@ -1016,7 +1021,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>38</v>
       </c>
@@ -1027,7 +1032,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>40</v>
       </c>
@@ -1038,7 +1043,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>41</v>
       </c>
@@ -1048,8 +1053,11 @@
       <c r="C38" s="8" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D38" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>42</v>
       </c>
@@ -1060,7 +1068,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="3">
         <v>43</v>
       </c>
@@ -1071,7 +1079,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="3">
         <v>44</v>
       </c>
@@ -1082,7 +1090,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
         <v>46</v>
       </c>
@@ -1093,7 +1101,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="3">
         <v>47</v>
       </c>
@@ -1105,6 +1113,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D38" r:id="rId1" xr:uid="{2FF02044-7ACD-490D-BD91-44A1DBBF2B13}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>